<commit_message>
incorporated the latest comments from SMEs
</commit_message>
<xml_diff>
--- a/MASTER.xlsx
+++ b/MASTER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javid Shiriyev\Documents\GitHub\sand-control-failure-db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086EEF7A-3267-436D-85F1-0191B958F2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8EB2284-67C5-423E-99C3-4528B8C90A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-2730" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterView" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1106" uniqueCount="413">
   <si>
     <t>Category</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Additional Bridging Agent</t>
   </si>
   <si>
-    <t>PSD Test Volume</t>
-  </si>
-  <si>
     <t>L</t>
   </si>
   <si>
@@ -698,9 +695,6 @@
     <t>Particle-size distribution of solids/bridging material in the reservoir drilling fluid.</t>
   </si>
   <si>
-    <t>Fluid or sample volume used to determine the reported drilling-fluid particle-size distribution.</t>
-  </si>
-  <si>
     <t>Primary completion configuration used across the production interval</t>
   </si>
   <si>
@@ -1151,9 +1145,6 @@
     <t>{"List": {"options": ["16/20", "16/30", "20/40", "30/50", "40/60", "40/70", "35 Monomesh", "25 Monomesh", "40 Monomesh", "45 Monomesh"]}}</t>
   </si>
   <si>
-    <t>{"List": {"options": ["Brine", "Xanthan", "VES", "HES", "Oil Based"]}}</t>
-  </si>
-  <si>
     <t>{"List": {"options": ["Xlink Gel", "VES", "HEC"]}}</t>
   </si>
   <si>
@@ -1202,9 +1193,6 @@
     <t>{"List": {"required": True, "options": ["Surface Solids Samples", "ASD Response", "Surface Equipment Erosion"]}}</t>
   </si>
   <si>
-    <t>{"List": {"required": True, "options": ["Aggressive drawdown", "Screen plugging", "Water breakthrough", "Water hammer", "Hard shutdown", "Other", "Unknown"]}}</t>
-  </si>
-  <si>
     <t>{"List": {"required": True, "options": ["Flowing Unrestricted by Sand", "Flowing Restricted by Sand", "Shut-in Due to Sand", "Shut in due to reasons other than sand", "Not Producing"]}}</t>
   </si>
   <si>
@@ -1265,13 +1253,28 @@
     <t>{"SAS": {"Gravel Packing": False}, "Cased and Perforated": {"Liners and Screens": False, "Gravel Packing": False}}</t>
   </si>
   <si>
-    <t>{"OHGP": {"Placement Method", "% Pack through Shunts", "Carrier Fluid Type - OHGP", "Pack Efficiency Source", "Pack Efficiency Percentage", "ICD / AICD", "Did screens get to Target Setting Depth", "Return Percentage", "If screens ran in mud, was mud removed once screens on bottom?"}, "SAS": {"Fluid Type Left in OH at end of Completion", "ICD / AICD", "Did screens get to Target Setting Depth", "If screens ran in mud, was mud removed once screens on bottom?", "Blank pipe run across non-pay sections instead of screens?"}, "CHFP": {"Carrier Fluid Type - CHFP", "Full Pack from Log"}, "CHGP": {"Carrier Fluid Type - CHGP", "Perf Packing", "Return Percentage", "Pack Efficiency Source", "Pack Efficiency Percentage"}}</t>
-  </si>
-  <si>
     <t>{"Measurable": {"Sand production rate at first choke back", "Sand production rate at well shut-in due to sand", "Sand production rate at complete well failure"}}</t>
   </si>
   <si>
     <t>At least 7 alphanumeric characters (letters/numbers only). Do not use the actual API/UWI number.</t>
+  </si>
+  <si>
+    <t>PST Test Volume</t>
+  </si>
+  <si>
+    <t>Volume of wellbore fluid sample passed through the screen coupon to ensure no plugging</t>
+  </si>
+  <si>
+    <t>{"List": {"options": ["Brine", "Xanthan", "VES", "HEC", "Oil Based"]}}</t>
+  </si>
+  <si>
+    <t>{"Shunt": {"% Pack through Shunts", "Shunt Tubes"}, "Circ Pack": {"% Pack through Shunts": False, "Shunt Tubes": False}}</t>
+  </si>
+  <si>
+    <t>{"OHGP": {"Placement Method", "Carrier Fluid Type - OHGP", "Pack Efficiency Source", "Pack Efficiency Percentage", "ICD / AICD", "Did screens get to Target Setting Depth", "Return Percentage", "If screens ran in mud, was mud removed once screens on bottom?"}, "SAS": {"Fluid Type Left in OH at end of Completion", "ICD / AICD", "Did screens get to Target Setting Depth", "If screens ran in mud, was mud removed once screens on bottom?", "Blank pipe run across non-pay sections instead of screens?"}, "CHFP": {"Carrier Fluid Type - CHFP", "Full Pack from Log"}, "CHGP": {"Carrier Fluid Type - CHGP", "Perf Packing", "Return Percentage", "Pack Efficiency Source", "Pack Efficiency Percentage"}}</t>
+  </si>
+  <si>
+    <t>{"List": {"required": True, "options": ["Aggressive Drawdown", "Screen Plugging", "Water Breakthrough", "Hard Shutdown", "Flux", "Incomplete Gravel Pack", "Compaction", "Excessive Drawdown", "Rapid Beanup", "Hard Shut-in", "Well Slugging", "Intervention Induced Damage", "Wrongly Sized Sand Control", "No Sand Control Installed", "Other", "Unknown"]}}</t>
   </si>
 </sst>
 </file>
@@ -2086,7 +2089,7 @@
     <col min="1" max="1" width="6.08984375" style="1" customWidth="1"/>
     <col min="2" max="2" width="6.90625" style="2" customWidth="1"/>
     <col min="3" max="3" width="9.81640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" customWidth="1"/>
+    <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="62.54296875" style="3" customWidth="1"/>
     <col min="7" max="7" width="14" style="2" customWidth="1"/>
     <col min="8" max="8" width="26.7265625" style="1" customWidth="1"/>
@@ -2100,7 +2103,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>3</v>
@@ -2130,10 +2133,10 @@
         <v>6</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="M1" s="1"/>
     </row>
@@ -2151,7 +2154,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>12</v>
@@ -2160,10 +2163,10 @@
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L2" s="5"/>
       <c r="M2" s="1"/>
@@ -2182,7 +2185,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>12</v>
@@ -2191,10 +2194,10 @@
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="1"/>
@@ -2213,7 +2216,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>13</v>
@@ -2222,10 +2225,10 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="J4" s="5" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L4" s="5"/>
       <c r="M4" s="1"/>
@@ -2244,7 +2247,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>13</v>
@@ -2253,10 +2256,10 @@
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
       <c r="J5" s="6" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L5" s="6"/>
       <c r="M5" s="1"/>
@@ -2275,7 +2278,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>13</v>
@@ -2284,10 +2287,10 @@
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
       <c r="J6" s="6" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="L6" s="6"/>
       <c r="M6" s="1"/>
@@ -2306,7 +2309,7 @@
         <v>15</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>12</v>
@@ -2314,13 +2317,13 @@
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L7" s="6"/>
       <c r="M7" s="1"/>
@@ -2339,7 +2342,7 @@
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>12</v>
@@ -2347,13 +2350,13 @@
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
       <c r="I8" s="6" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L8" s="6"/>
       <c r="M8" s="1"/>
@@ -2372,7 +2375,7 @@
         <v>15</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>16</v>
@@ -2383,10 +2386,10 @@
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="L9" s="6"/>
       <c r="M9" s="1"/>
@@ -2405,7 +2408,7 @@
         <v>15</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>12</v>
@@ -2414,10 +2417,10 @@
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="6" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L10" s="6"/>
       <c r="M10" s="1"/>
@@ -2447,10 +2450,10 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L11" s="6"/>
       <c r="M11" s="1"/>
@@ -2469,7 +2472,7 @@
         <v>15</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>16</v>
@@ -2480,10 +2483,10 @@
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="L12" s="6"/>
       <c r="M12" s="1"/>
@@ -2502,7 +2505,7 @@
         <v>15</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>13</v>
@@ -2511,10 +2514,10 @@
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L13" s="6"/>
       <c r="M13" s="1"/>
@@ -2533,7 +2536,7 @@
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>13</v>
@@ -2542,10 +2545,10 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L14" s="6"/>
       <c r="M14" s="1"/>
@@ -2564,7 +2567,7 @@
         <v>15</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>12</v>
@@ -2573,10 +2576,10 @@
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L15" s="6"/>
       <c r="M15" s="1"/>
@@ -2604,10 +2607,10 @@
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
       <c r="J16" s="6" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L16" s="6"/>
       <c r="M16" s="1"/>
@@ -2623,24 +2626,24 @@
         <v>14</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="6" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="L17" s="6"/>
       <c r="M17" s="1"/>
@@ -2659,7 +2662,7 @@
         <v>20</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>12</v>
@@ -2668,10 +2671,10 @@
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
       <c r="J18" s="6" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="L18" s="6"/>
       <c r="M18" s="1"/>
@@ -2690,7 +2693,7 @@
         <v>20</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>12</v>
@@ -2699,10 +2702,10 @@
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
       <c r="J19" s="6" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="L19" s="6"/>
       <c r="M19" s="1"/>
@@ -2721,7 +2724,7 @@
         <v>20</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>16</v>
@@ -2732,10 +2735,10 @@
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
       <c r="J20" s="6" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="L20" s="6"/>
       <c r="M20" s="1"/>
@@ -2754,7 +2757,7 @@
         <v>20</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>16</v>
@@ -2765,10 +2768,10 @@
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L21" s="6"/>
       <c r="M21" s="1"/>
@@ -2787,7 +2790,7 @@
         <v>20</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>16</v>
@@ -2798,10 +2801,10 @@
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="6" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L22" s="6"/>
       <c r="M22" s="1"/>
@@ -2820,7 +2823,7 @@
         <v>20</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>12</v>
@@ -2829,10 +2832,10 @@
       <c r="H23" s="6"/>
       <c r="I23" s="6"/>
       <c r="J23" s="6" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L23" s="6"/>
       <c r="M23" s="1"/>
@@ -2851,7 +2854,7 @@
         <v>20</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>12</v>
@@ -2860,10 +2863,10 @@
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
       <c r="J24" s="6" t="s">
-        <v>388</v>
+        <v>412</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L24" s="6"/>
       <c r="M24" s="1"/>
@@ -2882,7 +2885,7 @@
         <v>20</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>12</v>
@@ -2890,13 +2893,13 @@
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
       <c r="I25" s="6" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L25" s="6"/>
       <c r="M25" s="1"/>
@@ -2915,7 +2918,7 @@
         <v>20</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>16</v>
@@ -2926,10 +2929,10 @@
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
       <c r="J26" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L26" s="6"/>
       <c r="M26" s="1"/>
@@ -2948,7 +2951,7 @@
         <v>20</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>16</v>
@@ -2959,10 +2962,10 @@
       <c r="H27" s="6"/>
       <c r="I27" s="6"/>
       <c r="J27" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="L27" s="6"/>
       <c r="M27" s="1"/>
@@ -2981,7 +2984,7 @@
         <v>20</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>16</v>
@@ -2992,10 +2995,10 @@
       <c r="H28" s="6"/>
       <c r="I28" s="6"/>
       <c r="J28" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L28" s="6"/>
       <c r="M28" s="1"/>
@@ -3014,7 +3017,7 @@
         <v>20</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>16</v>
@@ -3025,10 +3028,10 @@
       <c r="H29" s="6"/>
       <c r="I29" s="6"/>
       <c r="J29" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="L29" s="6"/>
       <c r="M29" s="1"/>
@@ -3047,7 +3050,7 @@
         <v>20</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>16</v>
@@ -3056,10 +3059,10 @@
       <c r="H30" s="6"/>
       <c r="I30" s="6"/>
       <c r="J30" s="6" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="L30" s="6"/>
       <c r="M30" s="1"/>
@@ -3078,7 +3081,7 @@
         <v>20</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>16</v>
@@ -3087,10 +3090,10 @@
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
       <c r="J31" s="6" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L31" s="6"/>
       <c r="M31" s="1"/>
@@ -3109,7 +3112,7 @@
         <v>20</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>16</v>
@@ -3118,10 +3121,10 @@
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
       <c r="J32" s="6" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L32" s="6"/>
       <c r="M32" s="1"/>
@@ -3140,7 +3143,7 @@
         <v>20</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>16</v>
@@ -3151,10 +3154,10 @@
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L33" s="6"/>
       <c r="M33" s="1"/>
@@ -3173,7 +3176,7 @@
         <v>20</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>16</v>
@@ -3182,10 +3185,10 @@
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="L34" s="6"/>
       <c r="M34" s="1"/>
@@ -3204,7 +3207,7 @@
         <v>20</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F35" s="6" t="s">
         <v>16</v>
@@ -3213,10 +3216,10 @@
       <c r="H35" s="6"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L35" s="6"/>
       <c r="M35" s="1"/>
@@ -3235,7 +3238,7 @@
         <v>20</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>16</v>
@@ -3244,10 +3247,10 @@
       <c r="H36" s="6"/>
       <c r="I36" s="6"/>
       <c r="J36" s="6" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L36" s="6"/>
       <c r="M36" s="1"/>
@@ -3275,10 +3278,10 @@
       <c r="H37" s="6"/>
       <c r="I37" s="6"/>
       <c r="J37" s="6" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L37" s="6"/>
       <c r="M37" s="1"/>
@@ -3294,10 +3297,10 @@
         <v>14</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>12</v>
@@ -3306,10 +3309,10 @@
       <c r="H38" s="6"/>
       <c r="I38" s="6"/>
       <c r="J38" s="6" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L38" s="6"/>
       <c r="M38" s="1"/>
@@ -3325,10 +3328,10 @@
         <v>14</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="F39" s="6" t="s">
         <v>24</v>
@@ -3337,10 +3340,10 @@
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
       <c r="J39" s="6" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L39" s="6"/>
       <c r="M39" s="1"/>
@@ -3356,10 +3359,10 @@
         <v>14</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>24</v>
@@ -3368,10 +3371,10 @@
       <c r="H40" s="6"/>
       <c r="I40" s="6"/>
       <c r="J40" s="6" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L40" s="6"/>
       <c r="M40" s="1"/>
@@ -3387,10 +3390,10 @@
         <v>14</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="F41" s="6" t="s">
         <v>24</v>
@@ -3399,10 +3402,10 @@
       <c r="H41" s="6"/>
       <c r="I41" s="6"/>
       <c r="J41" s="6" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="L41" s="6"/>
       <c r="M41" s="1"/>
@@ -3418,7 +3421,7 @@
         <v>14</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>25</v>
@@ -3432,10 +3435,10 @@
       <c r="H42" s="6"/>
       <c r="I42" s="6"/>
       <c r="J42" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="L42" s="6"/>
       <c r="M42" s="1"/>
@@ -3451,7 +3454,7 @@
         <v>14</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>27</v>
@@ -3465,10 +3468,10 @@
       <c r="H43" s="6"/>
       <c r="I43" s="6"/>
       <c r="J43" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L43" s="6"/>
       <c r="M43" s="1"/>
@@ -3484,7 +3487,7 @@
         <v>14</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>28</v>
@@ -3498,10 +3501,10 @@
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
       <c r="J44" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K44" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="L44" s="6"/>
       <c r="M44" s="1"/>
@@ -3517,7 +3520,7 @@
         <v>14</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>30</v>
@@ -3531,10 +3534,10 @@
       <c r="H45" s="6"/>
       <c r="I45" s="6"/>
       <c r="J45" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="L45" s="6"/>
       <c r="M45" s="1"/>
@@ -3550,7 +3553,7 @@
         <v>14</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>31</v>
@@ -3564,10 +3567,10 @@
       <c r="H46" s="6"/>
       <c r="I46" s="6"/>
       <c r="J46" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L46" s="6"/>
       <c r="M46" s="1"/>
@@ -3583,7 +3586,7 @@
         <v>14</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>32</v>
@@ -3597,10 +3600,10 @@
       <c r="H47" s="6"/>
       <c r="I47" s="6"/>
       <c r="J47" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L47" s="6"/>
       <c r="M47" s="1"/>
@@ -3616,10 +3619,10 @@
         <v>14</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>16</v>
@@ -3630,10 +3633,10 @@
       <c r="H48" s="6"/>
       <c r="I48" s="6"/>
       <c r="J48" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L48" s="6"/>
       <c r="M48" s="1"/>
@@ -3649,10 +3652,10 @@
         <v>14</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="F49" s="6" t="s">
         <v>16</v>
@@ -3663,10 +3666,10 @@
       <c r="H49" s="6"/>
       <c r="I49" s="6"/>
       <c r="J49" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L49" s="6"/>
       <c r="M49" s="1"/>
@@ -3682,10 +3685,10 @@
         <v>14</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>16</v>
@@ -3696,10 +3699,10 @@
       <c r="H50" s="6"/>
       <c r="I50" s="6"/>
       <c r="J50" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L50" s="6"/>
       <c r="M50" s="1"/>
@@ -3715,10 +3718,10 @@
         <v>14</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F51" s="6" t="s">
         <v>16</v>
@@ -3729,10 +3732,10 @@
       <c r="H51" s="6"/>
       <c r="I51" s="6"/>
       <c r="J51" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L51" s="6"/>
       <c r="M51" s="1"/>
@@ -3748,10 +3751,10 @@
         <v>14</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>13</v>
@@ -3760,10 +3763,10 @@
       <c r="H52" s="6"/>
       <c r="I52" s="6"/>
       <c r="J52" s="6" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="L52" s="6"/>
       <c r="M52" s="1"/>
@@ -3779,10 +3782,10 @@
         <v>14</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>16</v>
@@ -3793,10 +3796,10 @@
       <c r="H53" s="6"/>
       <c r="I53" s="6"/>
       <c r="J53" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="L53" s="6"/>
       <c r="M53" s="1"/>
@@ -3812,10 +3815,10 @@
         <v>14</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>16</v>
@@ -3826,10 +3829,10 @@
       <c r="H54" s="6"/>
       <c r="I54" s="6"/>
       <c r="J54" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="L54" s="6"/>
       <c r="M54" s="1"/>
@@ -3845,10 +3848,10 @@
         <v>14</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="F55" s="6" t="s">
         <v>12</v>
@@ -3857,10 +3860,10 @@
       <c r="H55" s="6"/>
       <c r="I55" s="6"/>
       <c r="J55" s="6" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L55" s="6"/>
       <c r="M55" s="1"/>
@@ -3876,10 +3879,10 @@
         <v>14</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>12</v>
@@ -3888,10 +3891,10 @@
       <c r="H56" s="6"/>
       <c r="I56" s="6"/>
       <c r="J56" s="6" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L56" s="6"/>
       <c r="M56" s="1"/>
@@ -3907,10 +3910,10 @@
         <v>14</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="F57" s="6" t="s">
         <v>12</v>
@@ -3919,10 +3922,10 @@
       <c r="H57" s="6"/>
       <c r="I57" s="6"/>
       <c r="J57" s="6" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L57" s="6"/>
       <c r="M57" s="1"/>
@@ -3938,10 +3941,10 @@
         <v>14</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>12</v>
@@ -3950,10 +3953,10 @@
       <c r="H58" s="6"/>
       <c r="I58" s="6"/>
       <c r="J58" s="6" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L58" s="6"/>
       <c r="M58" s="1"/>
@@ -3966,13 +3969,13 @@
         <v>11</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F59" s="12" t="s">
         <v>16</v>
@@ -3981,10 +3984,10 @@
       <c r="H59" s="12"/>
       <c r="I59" s="12"/>
       <c r="J59" s="12" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K59" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="L59" s="11"/>
       <c r="M59" s="1"/>
@@ -3994,16 +3997,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>16</v>
@@ -4012,10 +4015,10 @@
       <c r="H60" s="7"/>
       <c r="I60" s="7"/>
       <c r="J60" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K60" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="L60" s="7"/>
       <c r="M60" s="1"/>
@@ -4025,32 +4028,32 @@
         <v>60</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D61" s="7" t="s">
         <v>36</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G61" s="7"/>
       <c r="H61" s="7" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="I61" s="7" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="J61" s="7" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="K61" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="L61" s="7"/>
       <c r="M61" s="1"/>
@@ -4060,16 +4063,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>36</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>24</v>
@@ -4078,10 +4081,10 @@
       <c r="H62" s="7"/>
       <c r="I62" s="7"/>
       <c r="J62" s="7" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="K62" s="7" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="L62" s="7"/>
       <c r="M62" s="1"/>
@@ -4091,30 +4094,30 @@
         <v>62</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H63" s="7"/>
       <c r="I63" s="7"/>
       <c r="J63" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K63" s="7" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="L63" s="7"/>
       <c r="M63" s="1"/>
@@ -4124,30 +4127,30 @@
         <v>63</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D64" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E64" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E64" s="7" t="s">
+      <c r="F64" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G64" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="F64" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G64" s="7" t="s">
-        <v>77</v>
       </c>
       <c r="H64" s="7"/>
       <c r="I64" s="7"/>
       <c r="J64" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="L64" s="7"/>
       <c r="M64" s="1"/>
@@ -4157,16 +4160,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F65" s="7" t="s">
         <v>16</v>
@@ -4177,10 +4180,10 @@
       <c r="H65" s="7"/>
       <c r="I65" s="7"/>
       <c r="J65" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K65" s="9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="L65" s="7"/>
       <c r="M65" s="1"/>
@@ -4190,16 +4193,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F66" s="7" t="s">
         <v>16</v>
@@ -4210,10 +4213,10 @@
       <c r="H66" s="7"/>
       <c r="I66" s="7"/>
       <c r="J66" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="L66" s="7"/>
       <c r="M66" s="1"/>
@@ -4223,28 +4226,28 @@
         <v>66</v>
       </c>
       <c r="B67" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G67" s="7"/>
       <c r="H67" s="7"/>
       <c r="I67" s="7"/>
       <c r="J67" s="7" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="K67" s="7" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="L67" s="7"/>
       <c r="M67" s="1"/>
@@ -4254,25 +4257,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G68" s="7"/>
       <c r="H68" s="7"/>
       <c r="I68" s="7"/>
       <c r="J68" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
@@ -4283,16 +4286,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>16</v>
@@ -4301,10 +4304,10 @@
       <c r="H69" s="7"/>
       <c r="I69" s="7"/>
       <c r="J69" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K69" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="L69" s="7"/>
       <c r="M69" s="1"/>
@@ -4314,13 +4317,13 @@
         <v>69</v>
       </c>
       <c r="B70" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E70" s="7" t="s">
         <v>37</v>
@@ -4332,10 +4335,10 @@
       <c r="H70" s="7"/>
       <c r="I70" s="7"/>
       <c r="J70" s="7" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L70" s="7"/>
       <c r="M70" s="1"/>
@@ -4345,13 +4348,13 @@
         <v>70</v>
       </c>
       <c r="B71" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>38</v>
@@ -4365,10 +4368,10 @@
       <c r="H71" s="7"/>
       <c r="I71" s="7"/>
       <c r="J71" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="L71" s="7"/>
       <c r="M71" s="1"/>
@@ -4378,13 +4381,13 @@
         <v>71</v>
       </c>
       <c r="B72" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E72" s="7" t="s">
         <v>40</v>
@@ -4396,10 +4399,10 @@
       <c r="H72" s="7"/>
       <c r="I72" s="7"/>
       <c r="J72" s="7" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="L72" s="7"/>
       <c r="M72" s="1"/>
@@ -4409,13 +4412,13 @@
         <v>72</v>
       </c>
       <c r="B73" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>41</v>
@@ -4427,10 +4430,10 @@
       <c r="H73" s="7"/>
       <c r="I73" s="7"/>
       <c r="J73" s="7" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L73" s="7"/>
       <c r="M73" s="1"/>
@@ -4440,16 +4443,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="F74" s="7" t="s">
         <v>13</v>
@@ -4458,10 +4461,10 @@
       <c r="H74" s="7"/>
       <c r="I74" s="7"/>
       <c r="J74" s="7" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="L74" s="7"/>
       <c r="M74" s="1"/>
@@ -4471,30 +4474,30 @@
         <v>74</v>
       </c>
       <c r="B75" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E75" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="F75" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G75" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="F75" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G75" s="7" t="s">
-        <v>43</v>
       </c>
       <c r="H75" s="7"/>
       <c r="I75" s="7"/>
       <c r="J75" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K75" s="7" t="s">
-        <v>220</v>
+        <v>408</v>
       </c>
       <c r="L75" s="7"/>
       <c r="M75" s="1"/>
@@ -4504,30 +4507,30 @@
         <v>75</v>
       </c>
       <c r="B76" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D76" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E76" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E76" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="F76" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H76" s="7"/>
       <c r="I76" s="7"/>
       <c r="J76" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="L76" s="7"/>
       <c r="M76" s="1"/>
@@ -4537,16 +4540,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F77" s="7" t="s">
         <v>16</v>
@@ -4557,10 +4560,10 @@
       <c r="H77" s="7"/>
       <c r="I77" s="7"/>
       <c r="J77" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="L77" s="7"/>
       <c r="M77" s="1"/>
@@ -4570,16 +4573,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D78" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F78" s="7" t="s">
         <v>16</v>
@@ -4590,10 +4593,10 @@
       <c r="H78" s="7"/>
       <c r="I78" s="7"/>
       <c r="J78" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K78" s="7" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="L78" s="7"/>
       <c r="M78" s="1"/>
@@ -4603,30 +4606,30 @@
         <v>78</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F79" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H79" s="7"/>
       <c r="I79" s="7"/>
       <c r="J79" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K79" s="7" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="L79" s="7"/>
       <c r="M79" s="1"/>
@@ -4636,30 +4639,30 @@
         <v>79</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E80" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="F80" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G80" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="F80" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G80" s="7" t="s">
-        <v>87</v>
       </c>
       <c r="H80" s="7"/>
       <c r="I80" s="7"/>
       <c r="J80" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K80" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="L80" s="7"/>
       <c r="M80" s="1"/>
@@ -4669,16 +4672,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F81" s="7" t="s">
         <v>12</v>
@@ -4687,10 +4690,10 @@
       <c r="H81" s="7"/>
       <c r="I81" s="7"/>
       <c r="J81" s="7" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="K81" s="7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="L81" s="7"/>
       <c r="M81" s="1"/>
@@ -4700,16 +4703,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D82" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E82" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F82" s="7" t="s">
         <v>12</v>
@@ -4718,10 +4721,10 @@
       <c r="H82" s="7"/>
       <c r="I82" s="7"/>
       <c r="J82" s="7" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="K82" s="7" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L82" s="7"/>
       <c r="M82" s="1"/>
@@ -4731,16 +4734,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D83" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F83" s="7" t="s">
         <v>12</v>
@@ -4749,10 +4752,10 @@
       <c r="H83" s="7"/>
       <c r="I83" s="7"/>
       <c r="J83" s="7" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="L83" s="7"/>
       <c r="M83" s="1"/>
@@ -4762,16 +4765,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D84" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F84" s="7" t="s">
         <v>16</v>
@@ -4782,10 +4785,10 @@
       <c r="H84" s="7"/>
       <c r="I84" s="7"/>
       <c r="J84" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L84" s="7"/>
       <c r="M84" s="1"/>
@@ -4795,32 +4798,32 @@
         <v>84</v>
       </c>
       <c r="B85" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E85" s="7" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="F85" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G85" s="7"/>
       <c r="H85" s="7" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="I85" s="7" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J85" s="7" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="L85" s="7"/>
       <c r="M85" s="1"/>
@@ -4830,32 +4833,32 @@
         <v>85</v>
       </c>
       <c r="B86" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D86" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E86" s="7" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="F86" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G86" s="7"/>
       <c r="H86" s="7" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="I86" s="7" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J86" s="7" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="K86" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="L86" s="7"/>
       <c r="M86" s="1"/>
@@ -4865,16 +4868,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D87" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E87" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F87" s="7" t="s">
         <v>12</v>
@@ -4883,10 +4886,10 @@
       <c r="H87" s="7"/>
       <c r="I87" s="7"/>
       <c r="J87" s="7" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K87" s="7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="L87" s="7"/>
       <c r="M87" s="1"/>
@@ -4896,16 +4899,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D88" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E88" s="7" t="s">
         <v>92</v>
-      </c>
-      <c r="E88" s="7" t="s">
-        <v>93</v>
       </c>
       <c r="F88" s="7" t="s">
         <v>12</v>
@@ -4914,10 +4917,10 @@
       <c r="H88" s="7"/>
       <c r="I88" s="7"/>
       <c r="J88" s="7" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="L88" s="7"/>
       <c r="M88" s="1"/>
@@ -4927,28 +4930,28 @@
         <v>88</v>
       </c>
       <c r="B89" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G89" s="7"/>
       <c r="H89" s="7"/>
       <c r="I89" s="7"/>
       <c r="J89" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K89" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="L89" s="7"/>
       <c r="M89" s="1"/>
@@ -4958,30 +4961,30 @@
         <v>89</v>
       </c>
       <c r="B90" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D90" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E90" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="F90" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G90" s="7" t="s">
         <v>95</v>
-      </c>
-      <c r="F90" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G90" s="7" t="s">
-        <v>96</v>
       </c>
       <c r="H90" s="7"/>
       <c r="I90" s="7"/>
       <c r="J90" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="L90" s="7"/>
       <c r="M90" s="1"/>
@@ -4991,30 +4994,30 @@
         <v>90</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D91" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="F91" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G91" s="7" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H91" s="7"/>
       <c r="I91" s="7"/>
       <c r="J91" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K91" s="7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="L91" s="7"/>
       <c r="M91" s="1"/>
@@ -5024,30 +5027,30 @@
         <v>91</v>
       </c>
       <c r="B92" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D92" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F92" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G92" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H92" s="7"/>
       <c r="I92" s="7"/>
       <c r="J92" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K92" s="7" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L92" s="7"/>
       <c r="M92" s="1"/>
@@ -5057,16 +5060,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D93" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F93" s="7" t="s">
         <v>12</v>
@@ -5075,10 +5078,10 @@
       <c r="H93" s="7"/>
       <c r="I93" s="7"/>
       <c r="J93" s="7" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L93" s="7"/>
       <c r="M93" s="1"/>
@@ -5088,16 +5091,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D94" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="F94" s="7" t="s">
         <v>12</v>
@@ -5106,10 +5109,10 @@
       <c r="H94" s="19"/>
       <c r="I94" s="19"/>
       <c r="J94" s="7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="L94" s="7"/>
       <c r="M94" s="1"/>
@@ -5119,16 +5122,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F95" s="7" t="s">
         <v>12</v>
@@ -5137,10 +5140,10 @@
       <c r="H95" s="7"/>
       <c r="I95" s="7"/>
       <c r="J95" s="7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K95" s="7" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="L95" s="7"/>
       <c r="M95" s="1"/>
@@ -5150,28 +5153,28 @@
         <v>95</v>
       </c>
       <c r="B96" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D96" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E96" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F96" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G96" s="7"/>
       <c r="H96" s="7"/>
       <c r="I96" s="7"/>
       <c r="J96" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K96" s="7" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="L96" s="7"/>
       <c r="M96" s="1"/>
@@ -5181,25 +5184,25 @@
         <v>96</v>
       </c>
       <c r="B97" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D97" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E97" s="7" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="F97" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G97" s="7"/>
       <c r="H97" s="7"/>
       <c r="I97" s="7"/>
       <c r="J97" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K97" s="7"/>
       <c r="L97" s="7"/>
@@ -5210,25 +5213,25 @@
         <v>97</v>
       </c>
       <c r="B98" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D98" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F98" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G98" s="7"/>
       <c r="H98" s="7"/>
       <c r="I98" s="7"/>
       <c r="J98" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K98" s="7"/>
       <c r="L98" s="7"/>
@@ -5239,28 +5242,30 @@
         <v>98</v>
       </c>
       <c r="B99" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D99" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E99" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="E99" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G99" s="7"/>
       <c r="H99" s="7"/>
-      <c r="I99" s="7"/>
+      <c r="I99" s="7" t="s">
+        <v>410</v>
+      </c>
       <c r="J99" s="7" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="K99" s="7" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="L99" s="7"/>
       <c r="M99" s="1"/>
@@ -5270,16 +5275,16 @@
         <v>99</v>
       </c>
       <c r="B100" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D100" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F100" s="7" t="s">
         <v>16</v>
@@ -5290,7 +5295,7 @@
       <c r="H100" s="20"/>
       <c r="I100" s="20"/>
       <c r="J100" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K100" s="7"/>
       <c r="L100" s="7"/>
@@ -5301,25 +5306,25 @@
         <v>100</v>
       </c>
       <c r="B101" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D101" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G101" s="7"/>
       <c r="H101" s="7"/>
       <c r="I101" s="7"/>
       <c r="J101" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K101" s="7"/>
       <c r="L101" s="7"/>
@@ -5330,16 +5335,16 @@
         <v>101</v>
       </c>
       <c r="B102" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D102" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F102" s="7" t="s">
         <v>12</v>
@@ -5348,10 +5353,10 @@
       <c r="H102" s="7"/>
       <c r="I102" s="7"/>
       <c r="J102" s="7" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="K102" s="7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="L102" s="7"/>
       <c r="M102" s="1"/>
@@ -5361,16 +5366,16 @@
         <v>102</v>
       </c>
       <c r="B103" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D103" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E103" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F103" s="7" t="s">
         <v>12</v>
@@ -5379,10 +5384,10 @@
       <c r="H103" s="7"/>
       <c r="I103" s="7"/>
       <c r="J103" s="7" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="K103" s="7" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="L103" s="7"/>
       <c r="M103" s="1"/>
@@ -5392,30 +5397,30 @@
         <v>103</v>
       </c>
       <c r="B104" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D104" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E104" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F104" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G104" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="H104" s="7"/>
       <c r="I104" s="7"/>
       <c r="J104" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K104" s="7" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="L104" s="7"/>
       <c r="M104" s="1"/>
@@ -5425,16 +5430,16 @@
         <v>104</v>
       </c>
       <c r="B105" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D105" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E105" s="7" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F105" s="7" t="s">
         <v>12</v>
@@ -5443,10 +5448,10 @@
       <c r="H105" s="7"/>
       <c r="I105" s="7"/>
       <c r="J105" s="7" t="s">
-        <v>371</v>
+        <v>409</v>
       </c>
       <c r="K105" s="7" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L105" s="7"/>
       <c r="M105" s="1"/>
@@ -5456,16 +5461,16 @@
         <v>105</v>
       </c>
       <c r="B106" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D106" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F106" s="7" t="s">
         <v>12</v>
@@ -5474,10 +5479,10 @@
       <c r="H106" s="7"/>
       <c r="I106" s="7"/>
       <c r="J106" s="7" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="K106" s="7" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L106" s="7"/>
       <c r="M106" s="1"/>
@@ -5487,16 +5492,16 @@
         <v>106</v>
       </c>
       <c r="B107" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D107" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F107" s="7" t="s">
         <v>12</v>
@@ -5505,10 +5510,10 @@
       <c r="H107" s="7"/>
       <c r="I107" s="7"/>
       <c r="J107" s="7" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="K107" s="7" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L107" s="7"/>
       <c r="M107" s="1"/>
@@ -5518,16 +5523,16 @@
         <v>107</v>
       </c>
       <c r="B108" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D108" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F108" s="7" t="s">
         <v>16</v>
@@ -5538,10 +5543,10 @@
       <c r="H108" s="7"/>
       <c r="I108" s="7"/>
       <c r="J108" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K108" s="7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="L108" s="7"/>
       <c r="M108" s="1"/>
@@ -5551,27 +5556,27 @@
         <v>108</v>
       </c>
       <c r="B109" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D109" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E109" s="13" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F109" s="14" t="s">
         <v>16</v>
       </c>
       <c r="G109" s="14" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="H109" s="20"/>
       <c r="I109" s="20"/>
       <c r="J109" s="14" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K109" s="14"/>
       <c r="L109" s="14"/>
@@ -5582,30 +5587,30 @@
         <v>109</v>
       </c>
       <c r="B110" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D110" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E110" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F110" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G110" s="7" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H110" s="7"/>
       <c r="I110" s="7"/>
       <c r="J110" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K110" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L110" s="7"/>
       <c r="M110" s="1"/>
@@ -5615,30 +5620,30 @@
         <v>110</v>
       </c>
       <c r="B111" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D111" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E111" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F111" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G111" s="7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H111" s="7"/>
       <c r="I111" s="7"/>
       <c r="J111" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K111" s="7" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="L111" s="7"/>
       <c r="M111" s="1"/>
@@ -5648,16 +5653,16 @@
         <v>111</v>
       </c>
       <c r="B112" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D112" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E112" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F112" s="7" t="s">
         <v>16</v>
@@ -5668,10 +5673,10 @@
       <c r="H112" s="7"/>
       <c r="I112" s="7"/>
       <c r="J112" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K112" s="7" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="L112" s="7"/>
       <c r="M112" s="1"/>
@@ -5681,16 +5686,16 @@
         <v>112</v>
       </c>
       <c r="B113" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F113" s="7" t="s">
         <v>16</v>
@@ -5701,10 +5706,10 @@
       <c r="H113" s="7"/>
       <c r="I113" s="7"/>
       <c r="J113" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K113" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L113" s="7"/>
       <c r="M113" s="1"/>
@@ -5714,25 +5719,25 @@
         <v>113</v>
       </c>
       <c r="B114" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D114" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F114" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G114" s="7"/>
       <c r="H114" s="7"/>
       <c r="I114" s="7"/>
       <c r="J114" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K114" s="7"/>
       <c r="L114" s="7"/>
@@ -5743,16 +5748,16 @@
         <v>114</v>
       </c>
       <c r="B115" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D115" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E115" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F115" s="7" t="s">
         <v>12</v>
@@ -5760,13 +5765,13 @@
       <c r="G115" s="7"/>
       <c r="H115" s="7"/>
       <c r="I115" s="7" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="J115" s="7" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="K115" s="7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="L115" s="7"/>
       <c r="M115" s="1"/>
@@ -5776,16 +5781,16 @@
         <v>115</v>
       </c>
       <c r="B116" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D116" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E116" s="7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="F116" s="7" t="s">
         <v>16</v>
@@ -5796,10 +5801,10 @@
       <c r="H116" s="7"/>
       <c r="I116" s="7"/>
       <c r="J116" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K116" s="7" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="L116" s="7"/>
       <c r="M116" s="1"/>
@@ -5809,28 +5814,28 @@
         <v>116</v>
       </c>
       <c r="B117" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D117" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E117" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G117" s="7"/>
       <c r="H117" s="7"/>
       <c r="I117" s="7"/>
       <c r="J117" s="7" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K117" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L117" s="7"/>
       <c r="M117" s="1"/>
@@ -5840,16 +5845,16 @@
         <v>117</v>
       </c>
       <c r="B118" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E118" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="F118" s="15" t="s">
         <v>16</v>
@@ -5858,10 +5863,10 @@
       <c r="H118" s="15"/>
       <c r="I118" s="15"/>
       <c r="J118" s="15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K118" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="L118" s="15"/>
       <c r="M118" s="1"/>
@@ -5871,16 +5876,16 @@
         <v>118</v>
       </c>
       <c r="B119" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C119" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D119" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E119" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F119" s="17" t="s">
         <v>12</v>
@@ -5889,10 +5894,10 @@
       <c r="H119" s="17"/>
       <c r="I119" s="17"/>
       <c r="J119" s="17" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="K119" s="17" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="L119" s="17"/>
       <c r="M119" s="1"/>
@@ -5902,16 +5907,16 @@
         <v>119</v>
       </c>
       <c r="B120" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C120" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D120" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E120" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F120" s="17" t="s">
         <v>12</v>
@@ -5920,10 +5925,10 @@
       <c r="H120" s="17"/>
       <c r="I120" s="17"/>
       <c r="J120" s="17" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="K120" s="17" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="L120" s="17"/>
       <c r="M120" s="1"/>
@@ -5933,16 +5938,16 @@
         <v>120</v>
       </c>
       <c r="B121" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C121" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D121" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E121" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F121" s="17" t="s">
         <v>12</v>
@@ -5951,10 +5956,10 @@
       <c r="H121" s="17"/>
       <c r="I121" s="17"/>
       <c r="J121" s="17" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="K121" s="17" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="L121" s="17"/>
       <c r="M121" s="1"/>
@@ -5964,16 +5969,16 @@
         <v>121</v>
       </c>
       <c r="B122" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C122" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D122" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E122" s="17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F122" s="17" t="s">
         <v>16</v>
@@ -5984,10 +5989,10 @@
       <c r="H122" s="17"/>
       <c r="I122" s="17"/>
       <c r="J122" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K122" s="17" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L122" s="17"/>
       <c r="M122" s="1"/>
@@ -5997,16 +6002,16 @@
         <v>122</v>
       </c>
       <c r="B123" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C123" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D123" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="E123" s="17" t="s">
         <v>52</v>
-      </c>
-      <c r="D123" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="E123" s="17" t="s">
-        <v>53</v>
       </c>
       <c r="F123" s="17" t="s">
         <v>16</v>
@@ -6017,10 +6022,10 @@
       <c r="H123" s="17"/>
       <c r="I123" s="17"/>
       <c r="J123" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K123" s="17" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L123" s="17"/>
       <c r="M123" s="1"/>
@@ -6030,16 +6035,16 @@
         <v>123</v>
       </c>
       <c r="B124" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C124" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D124" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E124" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F124" s="17" t="s">
         <v>16</v>
@@ -6050,10 +6055,10 @@
       <c r="H124" s="17"/>
       <c r="I124" s="17"/>
       <c r="J124" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K124" s="17" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="L124" s="17"/>
       <c r="M124" s="1"/>
@@ -6063,16 +6068,16 @@
         <v>124</v>
       </c>
       <c r="B125" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C125" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D125" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E125" s="17" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F125" s="17" t="s">
         <v>16</v>
@@ -6083,10 +6088,10 @@
       <c r="H125" s="17"/>
       <c r="I125" s="17"/>
       <c r="J125" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K125" s="17" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="L125" s="17"/>
       <c r="M125" s="1"/>
@@ -6096,30 +6101,30 @@
         <v>125</v>
       </c>
       <c r="B126" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C126" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D126" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E126" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="F126" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G126" s="17" t="s">
         <v>55</v>
-      </c>
-      <c r="F126" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G126" s="17" t="s">
-        <v>56</v>
       </c>
       <c r="H126" s="17"/>
       <c r="I126" s="17"/>
       <c r="J126" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K126" s="17" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="L126" s="17"/>
       <c r="M126" s="1"/>
@@ -6129,16 +6134,16 @@
         <v>126</v>
       </c>
       <c r="B127" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C127" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D127" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E127" s="17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F127" s="17" t="s">
         <v>16</v>
@@ -6149,10 +6154,10 @@
       <c r="H127" s="17"/>
       <c r="I127" s="17"/>
       <c r="J127" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K127" s="17" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="L127" s="17"/>
       <c r="M127" s="1"/>
@@ -6162,16 +6167,16 @@
         <v>127</v>
       </c>
       <c r="B128" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C128" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D128" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E128" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F128" s="17" t="s">
         <v>16</v>
@@ -6182,10 +6187,10 @@
       <c r="H128" s="17"/>
       <c r="I128" s="17"/>
       <c r="J128" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K128" s="17" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="L128" s="17"/>
       <c r="M128" s="1"/>
@@ -6195,16 +6200,16 @@
         <v>128</v>
       </c>
       <c r="B129" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C129" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D129" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E129" s="17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F129" s="17" t="s">
         <v>16</v>
@@ -6213,10 +6218,10 @@
       <c r="H129" s="17"/>
       <c r="I129" s="17"/>
       <c r="J129" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K129" s="17" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="L129" s="17"/>
       <c r="M129" s="1"/>
@@ -6226,30 +6231,30 @@
         <v>129</v>
       </c>
       <c r="B130" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C130" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D130" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E130" s="17" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F130" s="17" t="s">
         <v>16</v>
       </c>
       <c r="G130" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H130" s="17"/>
       <c r="I130" s="17"/>
       <c r="J130" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K130" s="17" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="L130" s="17"/>
       <c r="M130" s="1"/>
@@ -6259,30 +6264,30 @@
         <v>130</v>
       </c>
       <c r="B131" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C131" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D131" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E131" s="17" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F131" s="17" t="s">
         <v>16</v>
       </c>
       <c r="G131" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H131" s="17"/>
       <c r="I131" s="17"/>
       <c r="J131" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K131" s="17" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="L131" s="17"/>
       <c r="M131" s="1"/>
@@ -6292,16 +6297,16 @@
         <v>131</v>
       </c>
       <c r="B132" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C132" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D132" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E132" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F132" s="17" t="s">
         <v>12</v>
@@ -6310,10 +6315,10 @@
       <c r="H132" s="17"/>
       <c r="I132" s="17"/>
       <c r="J132" s="17" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="K132" s="17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="L132" s="17"/>
       <c r="M132" s="1"/>
@@ -6323,16 +6328,16 @@
         <v>132</v>
       </c>
       <c r="B133" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C133" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D133" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E133" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F133" s="17" t="s">
         <v>12</v>
@@ -6341,10 +6346,10 @@
       <c r="H133" s="17"/>
       <c r="I133" s="17"/>
       <c r="J133" s="17" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="K133" s="17" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="L133" s="17"/>
       <c r="M133" s="1"/>
@@ -6354,30 +6359,30 @@
         <v>133</v>
       </c>
       <c r="B134" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C134" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D134" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E134" s="17" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="F134" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G134" s="17" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H134" s="17"/>
       <c r="I134" s="17"/>
       <c r="J134" s="17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="K134" s="17" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="L134" s="17"/>
       <c r="M134" s="1"/>
@@ -6387,16 +6392,16 @@
         <v>134</v>
       </c>
       <c r="B135" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C135" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D135" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E135" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F135" s="17" t="s">
         <v>16</v>
@@ -6407,10 +6412,10 @@
       <c r="H135" s="17"/>
       <c r="I135" s="17"/>
       <c r="J135" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K135" s="17" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="L135" s="17"/>
       <c r="M135" s="1"/>
@@ -6420,16 +6425,16 @@
         <v>135</v>
       </c>
       <c r="B136" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C136" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D136" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E136" s="17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F136" s="17" t="s">
         <v>16</v>
@@ -6440,10 +6445,10 @@
       <c r="H136" s="17"/>
       <c r="I136" s="17"/>
       <c r="J136" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K136" s="17" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="L136" s="17"/>
       <c r="M136" s="1"/>
@@ -6453,16 +6458,16 @@
         <v>136</v>
       </c>
       <c r="B137" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C137" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D137" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E137" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F137" s="17" t="s">
         <v>16</v>
@@ -6473,10 +6478,10 @@
       <c r="H137" s="17"/>
       <c r="I137" s="17"/>
       <c r="J137" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K137" s="17" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="L137" s="17"/>
       <c r="M137" s="1"/>
@@ -6486,30 +6491,30 @@
         <v>137</v>
       </c>
       <c r="B138" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C138" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D138" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E138" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="F138" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G138" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="F138" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G138" s="17" t="s">
-        <v>64</v>
       </c>
       <c r="H138" s="17"/>
       <c r="I138" s="17"/>
       <c r="J138" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K138" s="17" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="L138" s="17"/>
       <c r="M138" s="1"/>
@@ -6519,30 +6524,30 @@
         <v>138</v>
       </c>
       <c r="B139" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C139" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D139" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E139" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="F139" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G139" s="17" t="s">
         <v>65</v>
-      </c>
-      <c r="F139" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G139" s="17" t="s">
-        <v>66</v>
       </c>
       <c r="H139" s="17"/>
       <c r="I139" s="17"/>
       <c r="J139" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K139" s="17" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="L139" s="17"/>
       <c r="M139" s="1"/>
@@ -6552,30 +6557,30 @@
         <v>139</v>
       </c>
       <c r="B140" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C140" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D140" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E140" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F140" s="17" t="s">
         <v>16</v>
       </c>
       <c r="G140" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H140" s="17"/>
       <c r="I140" s="17"/>
       <c r="J140" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K140" s="17" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="L140" s="17"/>
       <c r="M140" s="1"/>
@@ -6585,16 +6590,16 @@
         <v>140</v>
       </c>
       <c r="B141" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C141" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D141" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E141" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F141" s="17" t="s">
         <v>16</v>
@@ -6603,10 +6608,10 @@
       <c r="H141" s="17"/>
       <c r="I141" s="17"/>
       <c r="J141" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K141" s="17" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="L141" s="17"/>
       <c r="M141" s="1"/>
@@ -6616,16 +6621,16 @@
         <v>141</v>
       </c>
       <c r="B142" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C142" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D142" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E142" s="17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F142" s="17" t="s">
         <v>12</v>
@@ -6634,10 +6639,10 @@
       <c r="H142" s="17"/>
       <c r="I142" s="17"/>
       <c r="J142" s="17" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="K142" s="17" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="L142" s="17"/>
       <c r="M142" s="1"/>
@@ -6647,16 +6652,16 @@
         <v>142</v>
       </c>
       <c r="B143" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C143" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D143" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E143" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F143" s="17" t="s">
         <v>16</v>
@@ -6665,10 +6670,10 @@
       <c r="H143" s="17"/>
       <c r="I143" s="17"/>
       <c r="J143" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K143" s="17" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L143" s="17"/>
       <c r="M143" s="1"/>
@@ -6678,30 +6683,30 @@
         <v>143</v>
       </c>
       <c r="B144" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C144" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D144" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E144" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="F144" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G144" s="17" t="s">
         <v>70</v>
-      </c>
-      <c r="F144" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G144" s="17" t="s">
-        <v>71</v>
       </c>
       <c r="H144" s="17"/>
       <c r="I144" s="17"/>
       <c r="J144" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K144" s="17" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="L144" s="17"/>
       <c r="M144" s="1"/>
@@ -6711,16 +6716,16 @@
         <v>144</v>
       </c>
       <c r="B145" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C145" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D145" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E145" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F145" s="17" t="s">
         <v>16</v>
@@ -6731,10 +6736,10 @@
       <c r="H145" s="17"/>
       <c r="I145" s="17"/>
       <c r="J145" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K145" s="17" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="L145" s="17"/>
       <c r="M145" s="1"/>
@@ -6744,30 +6749,30 @@
         <v>145</v>
       </c>
       <c r="B146" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C146" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D146" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E146" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F146" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G146" s="17" t="s">
         <v>73</v>
-      </c>
-      <c r="F146" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G146" s="17" t="s">
-        <v>74</v>
       </c>
       <c r="H146" s="17"/>
       <c r="I146" s="17"/>
       <c r="J146" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K146" s="17" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="L146" s="17"/>
       <c r="M146" s="1"/>
@@ -6777,16 +6782,16 @@
         <v>146</v>
       </c>
       <c r="B147" s="17" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C147" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D147" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E147" s="17" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="F147" s="17" t="s">
         <v>16</v>
@@ -6797,10 +6802,10 @@
       <c r="H147" s="17"/>
       <c r="I147" s="17"/>
       <c r="J147" s="17" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K147" s="17" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="L147" s="17"/>
       <c r="M147" s="1"/>

</xml_diff>